<commit_message>
R05 (em andamento): correções da revisão (proporção do resíduo na E4, T14/T16 ampliados, EOB implícito do PET-RS) e rascunhos dos textos do artigo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CWPuQS1EQNnCbSqHfPPCuA
</commit_message>
<xml_diff>
--- a/parametros/quadro_parametros_v04.xlsx
+++ b/parametros/quadro_parametros_v04.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ONS — Operador Nacional do Sistema Elétrico, cálculo sobre os três SEAMSE acima ((jun/2019 − dez/2018) + dez/2019); acesso 2026-10-16T15:56:25Z; nan)</t>
+          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ano civil 2019 = (jun/2019 − dez/2018) + dez/2019 = Síntese da Apuração Mensal dos Serviços e Encargos (SEAMSE), dezembro/2018, p. 8 do PDF, seção 4 "Encargos pagos pelos usuários", linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 10.576.544.162,01), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201812.pdf, SHA-256 bf15544642f1… ; SEAMSE, junho/2019, p. 8 do PDF, seção 4, linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 21.367.058.292,17), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201906.pdf, SHA-256 4f6593756800… ; SEAMSE, dezembro/2019, p. 7 do PDF, seção 4, linha "Total Encargos de Uso", coluna do acumulado do ciclo 19/20 (R$ 12.145.090.044,99), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201912.pdf, SHA-256 b67d328b3129…)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1812.1 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1812.1 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 88.1 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 88.1 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 18088.8 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 18088.8 mil t: a referência 18088.8 das instruções é a soma das parcelas já arredondadas (17329.1 + 759.7 = 18088.8); o valor exato é 18088.87 mil t (18088.9 arredondado), e é o que vai no valor_t); 'Não alocado' não entra</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Exploração de petróleo e gás natural (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 23499.2 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Exploração de petróleo e gás natural (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 23499.2 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1155.4 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1155.4 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ONS — Operador Nacional do Sistema Elétrico, cálculo sobre os três SEAMSE acima ((jun/2019 − dez/2018) + dez/2019); acesso 2026-10-16T15:56:25Z; nan) × participação de RS no VBP do S38 (0.060645)</t>
+          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ano civil 2019 = (jun/2019 − dez/2018) + dez/2019 = Síntese da Apuração Mensal dos Serviços e Encargos (SEAMSE), dezembro/2018, p. 8 do PDF, seção 4 "Encargos pagos pelos usuários", linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 10.576.544.162,01), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201812.pdf, SHA-256 bf15544642f1… ; SEAMSE, junho/2019, p. 8 do PDF, seção 4, linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 21.367.058.292,17), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201906.pdf, SHA-256 4f6593756800… ; SEAMSE, dezembro/2019, p. 7 do PDF, seção 4, linha "Total Encargos de Uso", coluna do acumulado do ciclo 19/20 (R$ 12.145.090.044,99), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201912.pdf, SHA-256 b67d328b3129…) × participação de RS no VBP do S38 (0.060645)</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ONS — Operador Nacional do Sistema Elétrico, cálculo sobre os três SEAMSE acima ((jun/2019 − dez/2018) + dez/2019); acesso 2026-10-16T15:56:25Z; nan) × participação de RB no VBP do S38 (0.939355)</t>
+          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ano civil 2019 = (jun/2019 − dez/2018) + dez/2019 = Síntese da Apuração Mensal dos Serviços e Encargos (SEAMSE), dezembro/2018, p. 8 do PDF, seção 4 "Encargos pagos pelos usuários", linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 10.576.544.162,01), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201812.pdf, SHA-256 bf15544642f1… ; SEAMSE, junho/2019, p. 8 do PDF, seção 4, linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 21.367.058.292,17), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201906.pdf, SHA-256 4f6593756800… ; SEAMSE, dezembro/2019, p. 7 do PDF, seção 4, linha "Total Encargos de Uso", coluna do acumulado do ciclo 19/20 (R$ 12.145.090.044,99), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201912.pdf, SHA-256 b67d328b3129…) × participação de RB no VBP do S38 (0.939355)</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ONS — Operador Nacional do Sistema Elétrico, cálculo sobre os três SEAMSE acima ((jun/2019 − dez/2018) + dez/2019); acesso 2026-10-16T15:56:25Z; nan) × participação de RS no VBP do S38 (0.060645)</t>
+          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ano civil 2019 = (jun/2019 − dez/2018) + dez/2019 = Síntese da Apuração Mensal dos Serviços e Encargos (SEAMSE), dezembro/2018, p. 8 do PDF, seção 4 "Encargos pagos pelos usuários", linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 10.576.544.162,01), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201812.pdf, SHA-256 bf15544642f1… ; SEAMSE, junho/2019, p. 8 do PDF, seção 4, linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 21.367.058.292,17), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201906.pdf, SHA-256 4f6593756800… ; SEAMSE, dezembro/2019, p. 7 do PDF, seção 4, linha "Total Encargos de Uso", coluna do acumulado do ciclo 19/20 (R$ 12.145.090.044,99), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201912.pdf, SHA-256 b67d328b3129…) × participação de RS no VBP do S38 (0.060645)</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ONS — Operador Nacional do Sistema Elétrico, cálculo sobre os três SEAMSE acima ((jun/2019 − dez/2018) + dez/2019); acesso 2026-10-16T15:56:25Z; nan) × participação de RB no VBP do S38 (0.939355)</t>
+          <t>D17: encargos de uso do sistema de transmissão faturados pelo ONS no ano civil de 2019 (SEAMSE dez/2018, jun/2019 e dez/2019); sem PIS/Pasep e Cofins; inclui o orçamento do ONS (ano civil 2019 = (jun/2019 − dez/2018) + dez/2019 = Síntese da Apuração Mensal dos Serviços e Encargos (SEAMSE), dezembro/2018, p. 8 do PDF, seção 4 "Encargos pagos pelos usuários", linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 10.576.544.162,01), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201812.pdf, SHA-256 bf15544642f1… ; SEAMSE, junho/2019, p. 8 do PDF, seção 4, linha "Total Encargos de Uso", coluna "Total Ciclo 18/19" (R$ 21.367.058.292,17), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201906.pdf, SHA-256 4f6593756800… ; SEAMSE, dezembro/2019, p. 7 do PDF, seção 4, linha "Total Encargos de Uso", coluna do acumulado do ciclo 19/20 (R$ 12.145.090.044,99), https://www.ons.org.br/AcervoDigitalDocumentosEPublicacoes/SEAMSE_201912.pdf, SHA-256 b67d328b3129…) × participação de RB no VBP do S38 (0.939355)</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1812.1 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1812.1 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 88.1 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 88.1 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 18088.8 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Refino de petróleo (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 18088.8 mil t: a referência 18088.8 das instruções é a soma das parcelas já arredondadas (17329.1 + 759.7 = 18088.8); o valor exato é 18088.87 mil t (18088.9 arredondado), e é o que vai no valor_t); 'Não alocado' não entra</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Exploração de petróleo e gás natural (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 23499.2 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Exploração de petróleo e gás natural (Produção de combustíveis + Geração de eletricidade › Produção de combustíveis) — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 23499.2 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>E4 (Rodada 05, Seção 3.2): Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1155.4 mil t); 'Não alocado' não entra</t>
+          <t>HIPÓTESE (E4, sensibilidade; Rodada 05, Seção 3.2): a conta-satélite da NEREUS incluiria no S38 estas emissões do SEEG (indício do diagnóstico NEREUS × SEEG, não prova); se elas já estiverem nos setores de destino, a E4 as conta duas vezes (no S19-RS, por exemplo) — Produção de carvão mineral e outros — SEEG 13.0, Dados nacionais, aba Dados (https://seeg.eco.br/wp-content/uploads/2025/12/Dados-nacionais-13.0.xlsx; SHA-256 21fc49654828cdb2eb63c104f06ba19d08b7dd81229fd9bf8972d80834aff350); recorte em dados/externos/seeg/seeg13_2019_recorte_energia_v04.csv; scripts/rodada05_diagnostico_seeg.py; regra da E4 = instruções da Rodada 05, Seção 3.2 (referência 1155.4 mil t: confere (arredondamento a 0.1 mil t)); 'Não alocado' não entra</t>
         </is>
       </c>
     </row>

</xml_diff>